<commit_message>
Client Web 29 Sep v1
</commit_message>
<xml_diff>
--- a/assetsHTML/Atchison/SAAWeightsandRanges.xlsx
+++ b/assetsHTML/Atchison/SAAWeightsandRanges.xlsx
@@ -1585,7 +1585,7 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{1AEA2529-1882-4793-AAF5-1ADAE1848266}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{FD4E575C-A68B-4976-8010-330B20840A87}"/>
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1597,5 +1597,5 @@
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{8C2FDFB5-ED34-4255-8ABA-D6BDC95DEDA8}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{891389D2-452F-40C5-84BB-8813F9E9B683}"/>
 </file>
</xml_diff>